<commit_message>
fix mdms data + add billing service schemas
</commit_message>
<xml_diff>
--- a/jupyter/dataloader/templates/mdms_schema.xlsx
+++ b/jupyter/dataloader/templates/mdms_schema.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t xml:space="preserve">uniqueId</t>
   </si>
@@ -285,6 +285,191 @@
   </si>
   <si>
     <t xml:space="preserve">{"id":"6f68a861-c6fa-4cd2-9239-a2b231d9c61a","tenantId":"st","code":"egov-hrms.EmployeeDepartment","description":"HRMS Employee Department ","definition":{"type":"object","$schema":"http://json-schema.org/draft-07/schema#","required":["code"],"x-unique":["code"],"properties":{"code":{"type":"string"},"active":{"type":"boolean"}}},"isActive":true,"auditDetails":{"createdBy":"d7867ef2-d046-4361-9a82-94c35c98416e","lastModifiedBy":"d7867ef2-d046-4361-9a82-94c35c98416e","createdTime":1717573078335,"lastModifiedTime":1717573078335}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BillingService.BusinessService</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+            "id": "740ca689-5aa7-4bf6-9058-5def4bf25713",
+            "tenantId": "kl",
+            "code": "BillingService.BusinessService",
+            "description": null,
+            "definition": {
+                "type": "object",
+                "$schema": "http://json-schema.org/draft-07/schema#",
+                "required": [
+                    "businessService",
+                    "code",
+                    "collectionModesNotAllowed",
+                    "partPaymentAllowed",
+                    "minAmountPayable",
+                    "isAdvanceAllowed",
+                    "demandUpdateTime",
+                    "isVoucherCreationEnabled",
+                    "billGineiURL"
+                ],
+                "x-unique": [
+                    "code"
+                ],
+                "properties": {
+                    "code": {
+                        "type": "string"
+                    },
+                    "billGineiURL": {
+                        "type": "string"
+                    },
+                    "businessService": {
+                        "type": "string"
+                    },
+                    "demandUpdateTime": {
+                        "type": "integer"
+                    },
+                    "isAdvanceAllowed": {
+                        "type": "boolean"
+                    },
+                    "minAmountPayable": {
+                        "type": "integer"
+                    },
+                    "partPaymentAllowed": {
+                        "type": "boolean"
+                    },
+                    "isVoucherCreationEnabled": {
+                        "type": "boolean"
+                    },
+                    "collectionModesNotAllowed": {
+                        "type": "array",
+                        "items": {
+                            "type": "string"
+                        }
+                    }
+                },
+                "additionalProperties": false
+            },
+            "isActive": true,
+            "auditDetails": {
+                "createdBy": "3059806b-3059-4724-8ae1-d3f4e12686ff",
+                "lastModifiedBy": "3059806b-3059-4724-8ae1-d3f4e12686ff",
+                "createdTime": 1721743891566,
+                "lastModifiedTime": 1721743891566
+            }
+        }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BillingService.TaxHeadMaster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+            "id": "f5039eb9-f099-432f-9469-693810e4ca66",
+            "tenantId": "kl",
+            "code": "BillingService.TaxHeadMaster",
+            "description": null,
+            "definition": {
+                "type": "object",
+                "$schema": "http://json-schema.org/draft-07/schema#",
+                "required": [
+                    "category",
+                    "service",
+                    "name",
+                    "code",
+                    "isDebit",
+                    "isActualDemand",
+                    "order",
+                    "isRequired"
+                ],
+                "x-unique": [
+                    "code"
+                ],
+                "properties": {
+                    "code": {
+                        "type": "string"
+                    },
+                    "name": {
+                        "type": "string"
+                    },
+                    "order": {
+                        "type": "string"
+                    },
+                    "isDebit": {
+                        "type": "boolean"
+                    },
+                    "service": {
+                        "type": "string"
+                    },
+                    "category": {
+                        "type": "string"
+                    },
+                    "isRequired": {
+                        "type": "boolean"
+                    },
+                    "isActualDemand": {
+                        "type": "boolean"
+                    }
+                },
+                "additionalProperties": false
+            },
+            "isActive": true,
+            "auditDetails": {
+                "createdBy": "3059806b-3059-4724-8ae1-d3f4e12686ff",
+                "lastModifiedBy": "3059806b-3059-4724-8ae1-d3f4e12686ff",
+                "createdTime": 1721743892237,
+                "lastModifiedTime": 1721743892237
+            }
+        }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BillingService.TaxPeriod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+            "id": "15b8c549-7210-4e13-8408-7146e03d14ab",
+            "tenantId": "kl",
+            "code": "BillingService.TaxPeriod",
+            "description": null,
+            "definition": {
+                "type": "object",
+                "$schema": "http://json-schema.org/draft-07/schema#",
+                "required": [
+                    "fromDate",
+                    "toDate",
+                    "periodCycle",
+                    "service",
+                    "code",
+                    "financialYear"
+                ],
+                "x-unique": [
+                    "code"
+                ],
+                "properties": {
+                    "code": {
+                        "type": "string"
+                    },
+                    "toDate": {
+                        "type": "integer"
+                    },
+                    "service": {
+                        "type": "string"
+                    },
+                    "fromDate": {
+                        "type": "integer"
+                    },
+                    "periodCycle": {
+                        "type": "string"
+                    },
+                    "financialYear": {
+                        "type": "string"
+                    }
+                },
+                "additionalProperties": false
+            },
+            "isActive": true,
+            "auditDetails": {
+                "createdBy": "3059806b-3059-4724-8ae1-d3f4e12686ff",
+                "lastModifiedBy": "3059806b-3059-4724-8ae1-d3f4e12686ff",
+                "createdTime": 1721743892582,
+                "lastModifiedTime": 1721743892582
+            }
+        }</t>
   </si>
 </sst>
 </file>
@@ -329,6 +514,7 @@
       <color rgb="FF6AAB73"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1029,17 +1215,29 @@
         <v>87</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
-    </row>
-    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4"/>
-      <c r="B46" s="4"/>
-    </row>
-    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4"/>
-      <c r="B47" s="4"/>
+    <row r="45" customFormat="false" ht="814.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="724.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="623.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4"/>

</xml_diff>